<commit_message>
fix: inline listing links, remove redundant columns, fix column widths
- Listing name is now a direct link; Map button inline in same cell
- Remove Platform/English/Listing link/Map columns (14→10 cols)
- th min-width per column so table stays readable without overflow
- XLSX updated to match new column schema

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/rooms.xlsx
+++ b/rooms.xlsx
@@ -464,23 +464,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N34"/>
+  <dimension ref="A1:L34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="7" max="7"/>
     <col width="26" customWidth="1" min="8" max="8"/>
-    <col width="24" customWidth="1" min="9" max="9"/>
-    <col width="46" customWidth="1" min="10" max="10"/>
-    <col width="22" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="40" customWidth="1" min="14" max="14"/>
+    <col width="50" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="42" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -505,65 +503,55 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Platform</t>
+          <t>Type</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Type</t>
+          <t>Monthly rent</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Monthly rent</t>
+          <t>Total /mo</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Total /mo (incl 관리비)</t>
+          <t>Deposit</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Deposit</t>
+          <t>Size</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Size</t>
+          <t>Station</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>Nearest station</t>
+          <t>Commute</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>Commute to KHU</t>
+          <t>Options</t>
         </is>
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>Options</t>
+          <t>Listing link</t>
         </is>
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Naver Map</t>
         </is>
       </c>
       <c r="L4" s="3" t="inlineStr">
-        <is>
-          <t>Listing link</t>
-        </is>
-      </c>
-      <c r="M4" s="3" t="inlineStr">
-        <is>
-          <t>Naver Map</t>
-        </is>
-      </c>
-      <c r="N4" s="3" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -577,65 +565,55 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>33m2</t>
+          <t>쉐어하우스</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>쉐어하우스</t>
+          <t>₩498,333 / mo  (₩115,000 / week)</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>₩498,333 / mo  (₩115,000 / week)</t>
+          <t>₩585,000 / mo</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>₩585,000 / mo</t>
+          <t>₩330,000</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>₩330,000</t>
+          <t>13 m²</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>13 m²</t>
+          <t>회기역, 외대앞역</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>회기역, 외대앞역</t>
+          <t>Hoegi Stn, ~15 min walk or bus to KHU</t>
         </is>
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>Hoegi Stn, ~15 min walk or bus to KHU</t>
-        </is>
-      </c>
-      <c r="J5" s="4" t="inlineStr">
-        <is>
           <t>Fridge, Washer, A/C, WiFi, Induction, Bed, all utilities included</t>
         </is>
       </c>
-      <c r="K5" s="4" t="inlineStr">
-        <is>
-          <t>Yes — English app, foreign card OK</t>
-        </is>
-      </c>
-      <c r="L5" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="M5" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="N5" s="4" t="inlineStr">
+      <c r="J5" s="5" t="inlineStr">
+        <is>
+          <t>Open link</t>
+        </is>
+      </c>
+      <c r="K5" s="5" t="inlineStr">
+        <is>
+          <t>Open link</t>
+        </is>
+      </c>
+      <c r="L5" s="4" t="inlineStr">
         <is>
           <t>Min 2 weeks. Short-stay OK. 관리비 ₩86,667/mo included in total.</t>
         </is>
@@ -649,65 +627,55 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>33m2</t>
+          <t>쉐어하우스</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>쉐어하우스</t>
+          <t>₩541,667 / mo  (₩125,000 / week)</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>₩541,667 / mo  (₩125,000 / week)</t>
+          <t>₩598,000 / mo</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>₩598,000 / mo</t>
+          <t>₩330,000</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>₩330,000</t>
+          <t>10 m²</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>10 m²</t>
+          <t>회기역, 외대앞역</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>회기역, 외대앞역</t>
+          <t>Hoegi Stn, ~15 min walk or bus to KHU</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>Hoegi Stn, ~15 min walk or bus to KHU</t>
-        </is>
-      </c>
-      <c r="J6" s="4" t="inlineStr">
-        <is>
           <t>Fridge, Washer, A/C, TV, WiFi, Gas range, Bed, all utilities included</t>
         </is>
       </c>
-      <c r="K6" s="4" t="inlineStr">
-        <is>
-          <t>Yes — English app, foreign card OK</t>
-        </is>
-      </c>
-      <c r="L6" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="M6" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="N6" s="4" t="inlineStr">
+      <c r="J6" s="5" t="inlineStr">
+        <is>
+          <t>Open link</t>
+        </is>
+      </c>
+      <c r="K6" s="5" t="inlineStr">
+        <is>
+          <t>Open link</t>
+        </is>
+      </c>
+      <c r="L6" s="4" t="inlineStr">
         <is>
           <t>Min 12 weeks. 관리비 ₩56,333/mo included in total.</t>
         </is>
@@ -721,65 +689,55 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>33m2</t>
+          <t>쉐어하우스</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>쉐어하우스</t>
+          <t>₩541,667 / mo  (₩125,000 / week)</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>₩541,667 / mo  (₩125,000 / week)</t>
+          <t>₩650,000 / mo</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>₩650,000 / mo</t>
+          <t>₩330,000</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>₩330,000</t>
+          <t>17 m²</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>17 m²</t>
+          <t>회기역, 외대앞역</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>회기역, 외대앞역</t>
+          <t>Hoegi Stn, ~15 min walk or bus to KHU</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>Hoegi Stn, ~15 min walk or bus to KHU</t>
-        </is>
-      </c>
-      <c r="J7" s="4" t="inlineStr">
-        <is>
           <t>Fridge, Washer, A/C, WiFi, Induction, Bed, all utilities included</t>
         </is>
       </c>
-      <c r="K7" s="4" t="inlineStr">
-        <is>
-          <t>Yes — English app, foreign card OK</t>
-        </is>
-      </c>
-      <c r="L7" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="M7" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="N7" s="4" t="inlineStr">
+      <c r="J7" s="5" t="inlineStr">
+        <is>
+          <t>Open link</t>
+        </is>
+      </c>
+      <c r="K7" s="5" t="inlineStr">
+        <is>
+          <t>Open link</t>
+        </is>
+      </c>
+      <c r="L7" s="4" t="inlineStr">
         <is>
           <t>Min 11 weeks. 관리비 ₩108,333/mo included in total.</t>
         </is>
@@ -793,65 +751,55 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>33m2</t>
+          <t>쉐어하우스</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>쉐어하우스</t>
+          <t>₩520,000 / mo  (₩120,000 / week)</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>₩520,000 / mo  (₩120,000 / week)</t>
+          <t>₩650,000 / mo</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>₩650,000 / mo</t>
+          <t>₩330,000</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>₩330,000</t>
+          <t>3 m²</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>3 m²</t>
+          <t>회기역</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>회기역</t>
+          <t>Hoegi Stn, ~15 min walk or bus to KHU</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>Hoegi Stn, ~15 min walk or bus to KHU</t>
-        </is>
-      </c>
-      <c r="J8" s="4" t="inlineStr">
-        <is>
           <t>Fridge, Washer, A/C, WiFi, Gas range, Bed, all utilities included</t>
         </is>
       </c>
-      <c r="K8" s="4" t="inlineStr">
-        <is>
-          <t>Yes — English app, foreign card OK</t>
-        </is>
-      </c>
-      <c r="L8" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="M8" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="N8" s="4" t="inlineStr">
+      <c r="J8" s="5" t="inlineStr">
+        <is>
+          <t>Open link</t>
+        </is>
+      </c>
+      <c r="K8" s="5" t="inlineStr">
+        <is>
+          <t>Open link</t>
+        </is>
+      </c>
+      <c r="L8" s="4" t="inlineStr">
         <is>
           <t>Min 1 week. Short-stay OK. 관리비 ₩130,000/mo included in total.</t>
         </is>
@@ -865,65 +813,55 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>33m2</t>
+          <t>쉐어하우스</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>쉐어하우스</t>
+          <t>₩606,667 / mo  (₩140,000 / week)</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>₩606,667 / mo  (₩140,000 / week)</t>
+          <t>₩693,334 / mo</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>₩693,334 / mo</t>
+          <t>₩330,000</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>₩330,000</t>
+          <t>20 m²</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>20 m²</t>
+          <t>회기역</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>회기역</t>
+          <t>Hoegi Stn, ~15 min walk or bus to KHU</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>Hoegi Stn, ~15 min walk or bus to KHU</t>
-        </is>
-      </c>
-      <c r="J9" s="4" t="inlineStr">
-        <is>
           <t>Fridge, Washer, A/C, WiFi, Gas range, Bed, all utilities included</t>
         </is>
       </c>
-      <c r="K9" s="4" t="inlineStr">
-        <is>
-          <t>Yes — English app, foreign card OK</t>
-        </is>
-      </c>
-      <c r="L9" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="M9" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="N9" s="4" t="inlineStr">
+      <c r="J9" s="5" t="inlineStr">
+        <is>
+          <t>Open link</t>
+        </is>
+      </c>
+      <c r="K9" s="5" t="inlineStr">
+        <is>
+          <t>Open link</t>
+        </is>
+      </c>
+      <c r="L9" s="4" t="inlineStr">
         <is>
           <t>Min 4 weeks. 관리비 ₩86,667/mo included in total.</t>
         </is>
@@ -937,65 +875,55 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>33m2</t>
+          <t>쉐어하우스</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>쉐어하우스</t>
+          <t>₩585,000 / mo  (₩135,000 / week)</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>₩585,000 / mo  (₩135,000 / week)</t>
+          <t>₩715,000 / mo</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>₩715,000 / mo</t>
+          <t>₩330,000</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>₩330,000</t>
+          <t>13 m²</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>13 m²</t>
+          <t>회기역, 외대앞역</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>회기역, 외대앞역</t>
+          <t>Hoegi Stn, ~15 min walk or bus to KHU</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>Hoegi Stn, ~15 min walk or bus to KHU</t>
-        </is>
-      </c>
-      <c r="J10" s="4" t="inlineStr">
-        <is>
           <t>Fridge, Washer, A/C, TV, WiFi, Gas range, Bed, all utilities included</t>
         </is>
       </c>
-      <c r="K10" s="4" t="inlineStr">
-        <is>
-          <t>Yes — English app, foreign card OK</t>
-        </is>
-      </c>
-      <c r="L10" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="M10" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="N10" s="4" t="inlineStr">
+      <c r="J10" s="5" t="inlineStr">
+        <is>
+          <t>Open link</t>
+        </is>
+      </c>
+      <c r="K10" s="5" t="inlineStr">
+        <is>
+          <t>Open link</t>
+        </is>
+      </c>
+      <c r="L10" s="4" t="inlineStr">
         <is>
           <t>Min 2 weeks. Short-stay OK. 관리비 ₩130,000/mo included in total.</t>
         </is>
@@ -1009,65 +937,55 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>33m2</t>
+          <t>쉐어하우스</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>쉐어하우스</t>
+          <t>₩628,333 / mo  (₩145,000 / week)</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>₩628,333 / mo  (₩145,000 / week)</t>
+          <t>₩736,666 / mo</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>₩736,666 / mo</t>
+          <t>₩330,000</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>₩330,000</t>
+          <t>7 m²</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>7 m²</t>
+          <t>회기역, 외대앞역</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>회기역, 외대앞역</t>
+          <t>Hoegi Stn, ~15 min walk or bus to KHU</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>Hoegi Stn, ~15 min walk or bus to KHU</t>
-        </is>
-      </c>
-      <c r="J11" s="4" t="inlineStr">
-        <is>
           <t>Fridge, Washer, A/C, WiFi, Induction, Bed, all utilities included</t>
         </is>
       </c>
-      <c r="K11" s="4" t="inlineStr">
-        <is>
-          <t>Yes — English app, foreign card OK</t>
-        </is>
-      </c>
-      <c r="L11" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="M11" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="N11" s="4" t="inlineStr">
+      <c r="J11" s="5" t="inlineStr">
+        <is>
+          <t>Open link</t>
+        </is>
+      </c>
+      <c r="K11" s="5" t="inlineStr">
+        <is>
+          <t>Open link</t>
+        </is>
+      </c>
+      <c r="L11" s="4" t="inlineStr">
         <is>
           <t>Min 11 weeks. 관리비 ₩108,333/mo included in total.</t>
         </is>
@@ -1081,65 +999,55 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>33m2</t>
+          <t>Furnished studio</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Furnished studio</t>
+          <t>₩736,667 / mo  (₩170,000 / week)</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>₩736,667 / mo  (₩170,000 / week)</t>
+          <t>₩736,667 / mo</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>₩736,667 / mo</t>
+          <t>₩330,000</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>₩330,000</t>
+          <t>13 m²</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>13 m²</t>
+          <t>회기역</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>회기역</t>
+          <t>Hoegi Stn, ~15 min walk or bus to KHU</t>
         </is>
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>Hoegi Stn, ~15 min walk or bus to KHU</t>
-        </is>
-      </c>
-      <c r="J12" s="4" t="inlineStr">
-        <is>
           <t>Fridge, Washer, A/C, WiFi, Gas range, Bed, all utilities included</t>
         </is>
       </c>
-      <c r="K12" s="4" t="inlineStr">
-        <is>
-          <t>Yes — English app, foreign card OK</t>
-        </is>
-      </c>
-      <c r="L12" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="M12" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="N12" s="4" t="inlineStr">
+      <c r="J12" s="5" t="inlineStr">
+        <is>
+          <t>Open link</t>
+        </is>
+      </c>
+      <c r="K12" s="5" t="inlineStr">
+        <is>
+          <t>Open link</t>
+        </is>
+      </c>
+      <c r="L12" s="4" t="inlineStr">
         <is>
           <t>Min 2 weeks. Short-stay OK.</t>
         </is>
@@ -1153,65 +1061,55 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>33m2</t>
+          <t>쉐어하우스</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>쉐어하우스</t>
+          <t>₩650,000 / mo  (₩150,000 / week)</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>₩650,000 / mo  (₩150,000 / week)</t>
+          <t>₩736,667 / mo</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>₩736,667 / mo</t>
+          <t>₩330,000</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>₩330,000</t>
+          <t>10 m²</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>10 m²</t>
+          <t>회기역, 외대앞역</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>회기역, 외대앞역</t>
+          <t>Hoegi Stn, ~15 min walk or bus to KHU</t>
         </is>
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>Hoegi Stn, ~15 min walk or bus to KHU</t>
-        </is>
-      </c>
-      <c r="J13" s="4" t="inlineStr">
-        <is>
           <t>Fridge, Washer, A/C, WiFi, Induction, Bed, all utilities included</t>
         </is>
       </c>
-      <c r="K13" s="4" t="inlineStr">
-        <is>
-          <t>Yes — English app, foreign card OK</t>
-        </is>
-      </c>
-      <c r="L13" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="M13" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="N13" s="4" t="inlineStr">
+      <c r="J13" s="5" t="inlineStr">
+        <is>
+          <t>Open link</t>
+        </is>
+      </c>
+      <c r="K13" s="5" t="inlineStr">
+        <is>
+          <t>Open link</t>
+        </is>
+      </c>
+      <c r="L13" s="4" t="inlineStr">
         <is>
           <t>Min 1 week. Short-stay OK. 관리비 ₩86,667/mo included in total.</t>
         </is>
@@ -1225,65 +1123,55 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>33m2</t>
+          <t>Furnished studio</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Furnished studio</t>
+          <t>₩736,667 / mo  (₩170,000 / week)</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>₩736,667 / mo  (₩170,000 / week)</t>
+          <t>₩780,000 / mo</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>₩780,000 / mo</t>
+          <t>₩330,000</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>₩330,000</t>
+          <t>17 m²</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>17 m²</t>
+          <t>회기역, 외대앞역</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>회기역, 외대앞역</t>
+          <t>Hoegi Stn, ~15 min walk or bus to KHU</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>Hoegi Stn, ~15 min walk or bus to KHU</t>
-        </is>
-      </c>
-      <c r="J14" s="4" t="inlineStr">
-        <is>
           <t>Fridge, Washer, A/C, TV, WiFi, Induction, Bed, water included</t>
         </is>
       </c>
-      <c r="K14" s="4" t="inlineStr">
-        <is>
-          <t>Yes — English app, foreign card OK</t>
-        </is>
-      </c>
-      <c r="L14" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="M14" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="N14" s="4" t="inlineStr">
+      <c r="J14" s="5" t="inlineStr">
+        <is>
+          <t>Open link</t>
+        </is>
+      </c>
+      <c r="K14" s="5" t="inlineStr">
+        <is>
+          <t>Open link</t>
+        </is>
+      </c>
+      <c r="L14" s="4" t="inlineStr">
         <is>
           <t>Min 2 weeks. Short-stay OK. 관리비 ₩43,333/mo included in total.</t>
         </is>
@@ -1297,65 +1185,55 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>33m2</t>
+          <t>쉐어하우스</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>쉐어하우스</t>
+          <t>₩650,000 / mo  (₩150,000 / week)</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>₩650,000 / mo  (₩150,000 / week)</t>
+          <t>₩780,000 / mo</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>₩780,000 / mo</t>
+          <t>₩330,000</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>₩330,000</t>
+          <t>13 m²</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>13 m²</t>
+          <t>회기역, 외대앞역</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>회기역, 외대앞역</t>
+          <t>Hoegi Stn, ~15 min walk or bus to KHU</t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>Hoegi Stn, ~15 min walk or bus to KHU</t>
-        </is>
-      </c>
-      <c r="J15" s="4" t="inlineStr">
-        <is>
           <t>Fridge, Washer, A/C, WiFi, Gas range, Induction, Bed, all utilities included</t>
         </is>
       </c>
-      <c r="K15" s="4" t="inlineStr">
-        <is>
-          <t>Yes — English app, foreign card OK</t>
-        </is>
-      </c>
-      <c r="L15" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="M15" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="N15" s="4" t="inlineStr">
+      <c r="J15" s="5" t="inlineStr">
+        <is>
+          <t>Open link</t>
+        </is>
+      </c>
+      <c r="K15" s="5" t="inlineStr">
+        <is>
+          <t>Open link</t>
+        </is>
+      </c>
+      <c r="L15" s="4" t="inlineStr">
         <is>
           <t>Min 1 week. Short-stay OK. 관리비 ₩130,000/mo included in total.</t>
         </is>
@@ -1369,65 +1247,55 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>33m2</t>
+          <t>쉐어하우스</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>쉐어하우스</t>
+          <t>₩650,000 / mo  (₩150,000 / week)</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>₩650,000 / mo  (₩150,000 / week)</t>
+          <t>₩780,000 / mo</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>₩780,000 / mo</t>
+          <t>₩330,000</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>₩330,000</t>
+          <t>7 m²</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>7 m²</t>
+          <t>회기역</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>회기역</t>
+          <t>Hoegi Stn, ~15 min walk or bus to KHU</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>Hoegi Stn, ~15 min walk or bus to KHU</t>
-        </is>
-      </c>
-      <c r="J16" s="4" t="inlineStr">
-        <is>
           <t>Fridge, Washer, A/C, WiFi, Gas range, Bed, all utilities included</t>
         </is>
       </c>
-      <c r="K16" s="4" t="inlineStr">
-        <is>
-          <t>Yes — English app, foreign card OK</t>
-        </is>
-      </c>
-      <c r="L16" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="M16" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="N16" s="4" t="inlineStr">
+      <c r="J16" s="5" t="inlineStr">
+        <is>
+          <t>Open link</t>
+        </is>
+      </c>
+      <c r="K16" s="5" t="inlineStr">
+        <is>
+          <t>Open link</t>
+        </is>
+      </c>
+      <c r="L16" s="4" t="inlineStr">
         <is>
           <t>Min 1 week. Short-stay OK. 관리비 ₩130,000/mo included in total.</t>
         </is>
@@ -1441,65 +1309,55 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>33m2</t>
+          <t>쉐어하우스</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>쉐어하우스</t>
+          <t>₩693,333 / mo  (₩160,000 / week)</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>₩693,333 / mo  (₩160,000 / week)</t>
+          <t>₩801,666 / mo</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>₩801,666 / mo</t>
+          <t>₩330,000</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>₩330,000</t>
+          <t>10 m²</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>10 m²</t>
+          <t>회기역, 외대앞역</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>회기역, 외대앞역</t>
+          <t>Hoegi Stn, ~15 min walk or bus to KHU</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>Hoegi Stn, ~15 min walk or bus to KHU</t>
-        </is>
-      </c>
-      <c r="J17" s="4" t="inlineStr">
-        <is>
           <t>Fridge, Washer, A/C, WiFi, Induction, Bed, all utilities included</t>
         </is>
       </c>
-      <c r="K17" s="4" t="inlineStr">
-        <is>
-          <t>Yes — English app, foreign card OK</t>
-        </is>
-      </c>
-      <c r="L17" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="M17" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="N17" s="4" t="inlineStr">
+      <c r="J17" s="5" t="inlineStr">
+        <is>
+          <t>Open link</t>
+        </is>
+      </c>
+      <c r="K17" s="5" t="inlineStr">
+        <is>
+          <t>Open link</t>
+        </is>
+      </c>
+      <c r="L17" s="4" t="inlineStr">
         <is>
           <t>Min 11 weeks. 관리비 ₩108,333/mo included in total.</t>
         </is>
@@ -1513,65 +1371,55 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>33m2</t>
+          <t>Furnished studio</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Furnished studio</t>
+          <t>₩780,000 / mo  (₩180,000 / week)</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>₩780,000 / mo  (₩180,000 / week)</t>
+          <t>₩823,333 / mo</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>₩823,333 / mo</t>
+          <t>₩330,000</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>₩330,000</t>
+          <t>20 m²</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>20 m²</t>
+          <t>외대앞역, 회기역</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>외대앞역, 회기역</t>
+          <t>Hoegi Stn, ~15 min walk or bus to KHU</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>Hoegi Stn, ~15 min walk or bus to KHU</t>
-        </is>
-      </c>
-      <c r="J18" s="4" t="inlineStr">
-        <is>
           <t>Fridge, Washer, A/C, WiFi, Induction, Bed, all utilities included</t>
         </is>
       </c>
-      <c r="K18" s="4" t="inlineStr">
-        <is>
-          <t>Yes — English app, foreign card OK</t>
-        </is>
-      </c>
-      <c r="L18" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="M18" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="N18" s="4" t="inlineStr">
+      <c r="J18" s="5" t="inlineStr">
+        <is>
+          <t>Open link</t>
+        </is>
+      </c>
+      <c r="K18" s="5" t="inlineStr">
+        <is>
+          <t>Open link</t>
+        </is>
+      </c>
+      <c r="L18" s="4" t="inlineStr">
         <is>
           <t>Min 1 week. Short-stay OK. 관리비 ₩43,333/mo included in total.</t>
         </is>
@@ -1585,65 +1433,55 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>33m2</t>
+          <t>Detached house</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Detached house</t>
+          <t>₩563,333 / mo  (₩130,000 / week)</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>₩563,333 / mo  (₩130,000 / week)</t>
+          <t>₩866,666 / mo</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>₩866,666 / mo</t>
+          <t>₩330,000</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>₩330,000</t>
+          <t>13 m²</t>
         </is>
       </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
-          <t>13 m²</t>
+          <t>회기역</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>회기역</t>
+          <t>Hoegi Stn, ~15 min walk or bus to KHU</t>
         </is>
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>Hoegi Stn, ~15 min walk or bus to KHU</t>
-        </is>
-      </c>
-      <c r="J19" s="4" t="inlineStr">
-        <is>
           <t>Fridge, Washer, A/C, WiFi, Induction, Bed, all utilities included</t>
         </is>
       </c>
-      <c r="K19" s="4" t="inlineStr">
-        <is>
-          <t>Yes — English app, foreign card OK</t>
-        </is>
-      </c>
-      <c r="L19" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="M19" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="N19" s="4" t="inlineStr">
+      <c r="J19" s="5" t="inlineStr">
+        <is>
+          <t>Open link</t>
+        </is>
+      </c>
+      <c r="K19" s="5" t="inlineStr">
+        <is>
+          <t>Open link</t>
+        </is>
+      </c>
+      <c r="L19" s="4" t="inlineStr">
         <is>
           <t>Min 2 weeks. Short-stay OK. 관리비 ₩303,333/mo included in total.</t>
         </is>
@@ -1657,65 +1495,55 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>33m2</t>
+          <t>Detached house</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Detached house</t>
+          <t>₩866,667 / mo  (₩200,000 / week)</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>₩866,667 / mo  (₩200,000 / week)</t>
+          <t>₩866,667 / mo</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>₩866,667 / mo</t>
+          <t>₩330,000</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>₩330,000</t>
+          <t>40 m²</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
-          <t>40 m²</t>
+          <t>회기역, 외대앞역</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>회기역, 외대앞역</t>
+          <t>Hoegi Stn, ~15 min walk or bus to KHU</t>
         </is>
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>Hoegi Stn, ~15 min walk or bus to KHU</t>
-        </is>
-      </c>
-      <c r="J20" s="4" t="inlineStr">
-        <is>
           <t>Fridge, Washer, A/C, TV, Induction, Bed, all utilities included</t>
         </is>
       </c>
-      <c r="K20" s="4" t="inlineStr">
-        <is>
-          <t>Yes — English app, foreign card OK</t>
-        </is>
-      </c>
-      <c r="L20" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="M20" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="N20" s="4" t="inlineStr">
+      <c r="J20" s="5" t="inlineStr">
+        <is>
+          <t>Open link</t>
+        </is>
+      </c>
+      <c r="K20" s="5" t="inlineStr">
+        <is>
+          <t>Open link</t>
+        </is>
+      </c>
+      <c r="L20" s="4" t="inlineStr">
         <is>
           <t>Min 1 week. Short-stay OK.</t>
         </is>
@@ -1729,65 +1557,55 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>33m2</t>
+          <t>쉐어하우스</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>쉐어하우스</t>
+          <t>₩650,000 / mo  (₩150,000 / week)</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>₩650,000 / mo  (₩150,000 / week)</t>
+          <t>₩866,667 / mo</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>₩866,667 / mo</t>
+          <t>₩330,000</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>₩330,000</t>
+          <t>17 m²</t>
         </is>
       </c>
       <c r="G21" s="4" t="inlineStr">
         <is>
-          <t>17 m²</t>
+          <t>외대앞역, 회기역</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>외대앞역, 회기역</t>
+          <t>Hoegi Stn, ~15 min walk or bus to KHU</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>Hoegi Stn, ~15 min walk or bus to KHU</t>
-        </is>
-      </c>
-      <c r="J21" s="4" t="inlineStr">
-        <is>
           <t>Fridge, Washer, A/C, WiFi, Gas range, Bed, all utilities included</t>
         </is>
       </c>
-      <c r="K21" s="4" t="inlineStr">
-        <is>
-          <t>Yes — English app, foreign card OK</t>
-        </is>
-      </c>
-      <c r="L21" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="M21" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="N21" s="4" t="inlineStr">
+      <c r="J21" s="5" t="inlineStr">
+        <is>
+          <t>Open link</t>
+        </is>
+      </c>
+      <c r="K21" s="5" t="inlineStr">
+        <is>
+          <t>Open link</t>
+        </is>
+      </c>
+      <c r="L21" s="4" t="inlineStr">
         <is>
           <t>Min 1 week. Short-stay OK. 관리비 ₩216,667/mo included in total.</t>
         </is>
@@ -1801,65 +1619,55 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>33m2</t>
+          <t>Detached house</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Detached house</t>
+          <t>₩736,667 / mo  (₩170,000 / week)</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>₩736,667 / mo  (₩170,000 / week)</t>
+          <t>₩888,334 / mo</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>₩888,334 / mo</t>
+          <t>₩330,000</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>₩330,000</t>
+          <t>20 m²</t>
         </is>
       </c>
       <c r="G22" s="4" t="inlineStr">
         <is>
-          <t>20 m²</t>
+          <t>회기역</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>회기역</t>
+          <t>Hoegi Stn, ~15 min walk or bus to KHU</t>
         </is>
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>Hoegi Stn, ~15 min walk or bus to KHU</t>
-        </is>
-      </c>
-      <c r="J22" s="4" t="inlineStr">
-        <is>
           <t>Fridge, Washer, A/C, Gas range, Bed, all utilities included</t>
         </is>
       </c>
-      <c r="K22" s="4" t="inlineStr">
-        <is>
-          <t>Yes — English app, foreign card OK</t>
-        </is>
-      </c>
-      <c r="L22" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="M22" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="N22" s="4" t="inlineStr">
+      <c r="J22" s="5" t="inlineStr">
+        <is>
+          <t>Open link</t>
+        </is>
+      </c>
+      <c r="K22" s="5" t="inlineStr">
+        <is>
+          <t>Open link</t>
+        </is>
+      </c>
+      <c r="L22" s="4" t="inlineStr">
         <is>
           <t>Min 1 week. Short-stay OK. 관리비 ₩151,667/mo included in total.</t>
         </is>
@@ -1873,65 +1681,55 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>33m2</t>
+          <t>쉐어하우스</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>쉐어하우스</t>
+          <t>₩780,000 / mo  (₩180,000 / week)</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>₩780,000 / mo  (₩180,000 / week)</t>
+          <t>₩910,000 / mo</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>₩910,000 / mo</t>
+          <t>₩330,000</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>₩330,000</t>
+          <t>7 m²</t>
         </is>
       </c>
       <c r="G23" s="4" t="inlineStr">
         <is>
-          <t>7 m²</t>
+          <t>회기역, 외대앞역</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t>회기역, 외대앞역</t>
+          <t>Hoegi Stn, ~15 min walk or bus to KHU</t>
         </is>
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>Hoegi Stn, ~15 min walk or bus to KHU</t>
-        </is>
-      </c>
-      <c r="J23" s="4" t="inlineStr">
-        <is>
           <t>Fridge, Washer, A/C, WiFi, Gas range, Induction, Bed, all utilities included</t>
         </is>
       </c>
-      <c r="K23" s="4" t="inlineStr">
-        <is>
-          <t>Yes — English app, foreign card OK</t>
-        </is>
-      </c>
-      <c r="L23" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="M23" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="N23" s="4" t="inlineStr">
+      <c r="J23" s="5" t="inlineStr">
+        <is>
+          <t>Open link</t>
+        </is>
+      </c>
+      <c r="K23" s="5" t="inlineStr">
+        <is>
+          <t>Open link</t>
+        </is>
+      </c>
+      <c r="L23" s="4" t="inlineStr">
         <is>
           <t>Min 1 week. Short-stay OK. 관리비 ₩130,000/mo included in total.</t>
         </is>
@@ -1945,65 +1743,55 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>33m2</t>
+          <t>Detached house</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Detached house</t>
+          <t>₩650,000 / mo  (₩150,000 / week)</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>₩650,000 / mo  (₩150,000 / week)</t>
+          <t>₩953,333 / mo</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>₩953,333 / mo</t>
+          <t>₩330,000</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>₩330,000</t>
+          <t>17 m²</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t>17 m²</t>
+          <t>회기역</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr">
         <is>
-          <t>회기역</t>
+          <t>Hoegi Stn, ~15 min walk or bus to KHU</t>
         </is>
       </c>
       <c r="I24" s="4" t="inlineStr">
         <is>
-          <t>Hoegi Stn, ~15 min walk or bus to KHU</t>
-        </is>
-      </c>
-      <c r="J24" s="4" t="inlineStr">
-        <is>
           <t>Fridge, Washer, A/C, WiFi, Gas range, Bed, all utilities included</t>
         </is>
       </c>
-      <c r="K24" s="4" t="inlineStr">
-        <is>
-          <t>Yes — English app, foreign card OK</t>
-        </is>
-      </c>
-      <c r="L24" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="M24" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="N24" s="4" t="inlineStr">
+      <c r="J24" s="5" t="inlineStr">
+        <is>
+          <t>Open link</t>
+        </is>
+      </c>
+      <c r="K24" s="5" t="inlineStr">
+        <is>
+          <t>Open link</t>
+        </is>
+      </c>
+      <c r="L24" s="4" t="inlineStr">
         <is>
           <t>Min 2 weeks. Short-stay OK. 관리비 ₩303,333/mo included in total.</t>
         </is>
@@ -2017,65 +1805,55 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>33m2</t>
+          <t>Detached house</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Detached house</t>
+          <t>₩650,000 / mo  (₩150,000 / week)</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>₩650,000 / mo  (₩150,000 / week)</t>
+          <t>₩953,333 / mo</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>₩953,333 / mo</t>
+          <t>₩330,000</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>₩330,000</t>
+          <t>20 m²</t>
         </is>
       </c>
       <c r="G25" s="4" t="inlineStr">
         <is>
-          <t>20 m²</t>
+          <t>회기역</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>회기역</t>
+          <t>Hoegi Stn, ~15 min walk or bus to KHU</t>
         </is>
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>Hoegi Stn, ~15 min walk or bus to KHU</t>
-        </is>
-      </c>
-      <c r="J25" s="4" t="inlineStr">
-        <is>
           <t>Fridge, Washer, A/C, WiFi, Induction, Bed, all utilities included</t>
         </is>
       </c>
-      <c r="K25" s="4" t="inlineStr">
-        <is>
-          <t>Yes — English app, foreign card OK</t>
-        </is>
-      </c>
-      <c r="L25" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="M25" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="N25" s="4" t="inlineStr">
+      <c r="J25" s="5" t="inlineStr">
+        <is>
+          <t>Open link</t>
+        </is>
+      </c>
+      <c r="K25" s="5" t="inlineStr">
+        <is>
+          <t>Open link</t>
+        </is>
+      </c>
+      <c r="L25" s="4" t="inlineStr">
         <is>
           <t>Min 2 weeks. Short-stay OK. 관리비 ₩303,333/mo included in total.</t>
         </is>
@@ -2089,65 +1867,55 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>33m2</t>
+          <t>Furnished studio</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Furnished studio</t>
+          <t>₩953,333 / mo  (₩220,000 / week)</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>₩953,333 / mo  (₩220,000 / week)</t>
+          <t>₩953,333 / mo</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>₩953,333 / mo</t>
+          <t>₩330,000</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>₩330,000</t>
+          <t>20 m²</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr">
         <is>
-          <t>20 m²</t>
+          <t>회기역</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr">
         <is>
-          <t>회기역</t>
+          <t>Hoegi Stn, ~15 min walk or bus to KHU</t>
         </is>
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>Hoegi Stn, ~15 min walk or bus to KHU</t>
-        </is>
-      </c>
-      <c r="J26" s="4" t="inlineStr">
-        <is>
           <t>Fridge, Washer, A/C, WiFi, Gas range, Bed, all utilities included</t>
         </is>
       </c>
-      <c r="K26" s="4" t="inlineStr">
-        <is>
-          <t>Yes — English app, foreign card OK</t>
-        </is>
-      </c>
-      <c r="L26" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="M26" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="N26" s="4" t="inlineStr">
+      <c r="J26" s="5" t="inlineStr">
+        <is>
+          <t>Open link</t>
+        </is>
+      </c>
+      <c r="K26" s="5" t="inlineStr">
+        <is>
+          <t>Open link</t>
+        </is>
+      </c>
+      <c r="L26" s="4" t="inlineStr">
         <is>
           <t>Min 2 weeks. Short-stay OK.</t>
         </is>
@@ -2161,65 +1929,55 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>33m2</t>
+          <t>쉐어하우스</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>쉐어하우스</t>
+          <t>₩975,000 / mo  (₩225,000 / week)</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>₩975,000 / mo  (₩225,000 / week)</t>
+          <t>₩975,000 / mo</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>₩975,000 / mo</t>
+          <t>₩330,000</t>
         </is>
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>₩330,000</t>
+          <t>10 m²</t>
         </is>
       </c>
       <c r="G27" s="4" t="inlineStr">
         <is>
-          <t>10 m²</t>
+          <t>회기역, 외대앞역</t>
         </is>
       </c>
       <c r="H27" s="4" t="inlineStr">
         <is>
-          <t>회기역, 외대앞역</t>
+          <t>Hoegi Stn, ~15 min walk or bus to KHU</t>
         </is>
       </c>
       <c r="I27" s="4" t="inlineStr">
         <is>
-          <t>Hoegi Stn, ~15 min walk or bus to KHU</t>
-        </is>
-      </c>
-      <c r="J27" s="4" t="inlineStr">
-        <is>
           <t>Fridge, Washer, A/C, WiFi, Induction, Bed, all utilities included</t>
         </is>
       </c>
-      <c r="K27" s="4" t="inlineStr">
-        <is>
-          <t>Yes — English app, foreign card OK</t>
-        </is>
-      </c>
-      <c r="L27" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="M27" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="N27" s="4" t="inlineStr">
+      <c r="J27" s="5" t="inlineStr">
+        <is>
+          <t>Open link</t>
+        </is>
+      </c>
+      <c r="K27" s="5" t="inlineStr">
+        <is>
+          <t>Open link</t>
+        </is>
+      </c>
+      <c r="L27" s="4" t="inlineStr">
         <is>
           <t>Min 1 week. Short-stay OK.</t>
         </is>
@@ -2233,65 +1991,55 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>33m2</t>
+          <t>Detached house</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>Detached house</t>
+          <t>₩693,333 / mo  (₩160,000 / week)</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>₩693,333 / mo  (₩160,000 / week)</t>
+          <t>₩996,666 / mo</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>₩996,666 / mo</t>
+          <t>₩330,000</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>₩330,000</t>
+          <t>20 m²</t>
         </is>
       </c>
       <c r="G28" s="4" t="inlineStr">
         <is>
-          <t>20 m²</t>
+          <t>회기역</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr">
         <is>
-          <t>회기역</t>
+          <t>Hoegi Stn, ~15 min walk or bus to KHU</t>
         </is>
       </c>
       <c r="I28" s="4" t="inlineStr">
         <is>
-          <t>Hoegi Stn, ~15 min walk or bus to KHU</t>
-        </is>
-      </c>
-      <c r="J28" s="4" t="inlineStr">
-        <is>
           <t>Fridge, Washer, A/C, WiFi, Induction, Bed, all utilities included</t>
         </is>
       </c>
-      <c r="K28" s="4" t="inlineStr">
-        <is>
-          <t>Yes — English app, foreign card OK</t>
-        </is>
-      </c>
-      <c r="L28" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="M28" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="N28" s="4" t="inlineStr">
+      <c r="J28" s="5" t="inlineStr">
+        <is>
+          <t>Open link</t>
+        </is>
+      </c>
+      <c r="K28" s="5" t="inlineStr">
+        <is>
+          <t>Open link</t>
+        </is>
+      </c>
+      <c r="L28" s="4" t="inlineStr">
         <is>
           <t>Min 2 weeks. Short-stay OK. 관리비 ₩303,333/mo included in total.</t>
         </is>
@@ -2305,65 +2053,55 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>33m2</t>
+          <t>쉐어하우스</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>쉐어하우스</t>
+          <t>₩866,667 / mo  (₩200,000 / week)</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>₩866,667 / mo  (₩200,000 / week)</t>
+          <t>₩996,667 / mo</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>₩996,667 / mo</t>
+          <t>₩330,000</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>₩330,000</t>
+          <t>17 m²</t>
         </is>
       </c>
       <c r="G29" s="4" t="inlineStr">
         <is>
-          <t>17 m²</t>
+          <t>회기역, 외대앞역</t>
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr">
         <is>
-          <t>회기역, 외대앞역</t>
+          <t>Hoegi Stn, ~15 min walk or bus to KHU</t>
         </is>
       </c>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t>Hoegi Stn, ~15 min walk or bus to KHU</t>
-        </is>
-      </c>
-      <c r="J29" s="4" t="inlineStr">
-        <is>
           <t>Fridge, Washer, A/C, WiFi, Gas range, Bed, all utilities included</t>
         </is>
       </c>
-      <c r="K29" s="4" t="inlineStr">
-        <is>
-          <t>Yes — English app, foreign card OK</t>
-        </is>
-      </c>
-      <c r="L29" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="M29" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="N29" s="4" t="inlineStr">
+      <c r="J29" s="5" t="inlineStr">
+        <is>
+          <t>Open link</t>
+        </is>
+      </c>
+      <c r="K29" s="5" t="inlineStr">
+        <is>
+          <t>Open link</t>
+        </is>
+      </c>
+      <c r="L29" s="4" t="inlineStr">
         <is>
           <t>Min 4 weeks. 관리비 ₩130,000/mo included in total.</t>
         </is>
@@ -2377,65 +2115,55 @@
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>33m2</t>
+          <t>쉐어하우스</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>쉐어하우스</t>
+          <t>₩736,667 / mo  (₩170,000 / week)</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>₩736,667 / mo  (₩170,000 / week)</t>
+          <t>₩996,667 / mo</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>₩996,667 / mo</t>
+          <t>₩330,000</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>₩330,000</t>
+          <t>17 m²</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr">
         <is>
-          <t>17 m²</t>
+          <t>외대앞역, 회기역</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr">
         <is>
-          <t>외대앞역, 회기역</t>
+          <t>Hoegi Stn, ~15 min walk or bus to KHU</t>
         </is>
       </c>
       <c r="I30" s="4" t="inlineStr">
         <is>
-          <t>Hoegi Stn, ~15 min walk or bus to KHU</t>
-        </is>
-      </c>
-      <c r="J30" s="4" t="inlineStr">
-        <is>
           <t>Fridge, Washer, A/C, WiFi, Gas range, Bed, all utilities included</t>
         </is>
       </c>
-      <c r="K30" s="4" t="inlineStr">
-        <is>
-          <t>Yes — English app, foreign card OK</t>
-        </is>
-      </c>
-      <c r="L30" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="M30" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="N30" s="4" t="inlineStr">
+      <c r="J30" s="5" t="inlineStr">
+        <is>
+          <t>Open link</t>
+        </is>
+      </c>
+      <c r="K30" s="5" t="inlineStr">
+        <is>
+          <t>Open link</t>
+        </is>
+      </c>
+      <c r="L30" s="4" t="inlineStr">
         <is>
           <t>Min 1 week. Short-stay OK. 관리비 ₩260,000/mo included in total.</t>
         </is>
@@ -2449,65 +2177,55 @@
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>33m2</t>
+          <t>쉐어하우스</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>쉐어하우스</t>
+          <t>₩910,000 / mo  (₩210,000 / week)</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>₩910,000 / mo  (₩210,000 / week)</t>
+          <t>₩1,040,000 / mo</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>₩1,040,000 / mo</t>
+          <t>₩330,000</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>₩330,000</t>
+          <t>10 m²</t>
         </is>
       </c>
       <c r="G31" s="4" t="inlineStr">
         <is>
-          <t>10 m²</t>
+          <t>회기역, 외대앞역</t>
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr">
         <is>
-          <t>회기역, 외대앞역</t>
+          <t>Hoegi Stn, ~15 min walk or bus to KHU</t>
         </is>
       </c>
       <c r="I31" s="4" t="inlineStr">
         <is>
-          <t>Hoegi Stn, ~15 min walk or bus to KHU</t>
-        </is>
-      </c>
-      <c r="J31" s="4" t="inlineStr">
-        <is>
           <t>Fridge, Washer, A/C, WiFi, Gas range, Induction, Bed, all utilities included</t>
         </is>
       </c>
-      <c r="K31" s="4" t="inlineStr">
-        <is>
-          <t>Yes — English app, foreign card OK</t>
-        </is>
-      </c>
-      <c r="L31" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="M31" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="N31" s="4" t="inlineStr">
+      <c r="J31" s="5" t="inlineStr">
+        <is>
+          <t>Open link</t>
+        </is>
+      </c>
+      <c r="K31" s="5" t="inlineStr">
+        <is>
+          <t>Open link</t>
+        </is>
+      </c>
+      <c r="L31" s="4" t="inlineStr">
         <is>
           <t>Min 1 week. Short-stay OK. 관리비 ₩130,000/mo included in total.</t>
         </is>
@@ -2521,65 +2239,55 @@
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>33m2</t>
+          <t>Furnished studio</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>Furnished studio</t>
+          <t>₩910,000 / mo  (₩210,000 / week)</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>₩910,000 / mo  (₩210,000 / week)</t>
+          <t>₩1,083,333 / mo</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>₩1,083,333 / mo</t>
+          <t>₩330,000</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>₩330,000</t>
+          <t>23 m²</t>
         </is>
       </c>
       <c r="G32" s="4" t="inlineStr">
         <is>
-          <t>23 m²</t>
+          <t>회기역, 외대앞역</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr">
         <is>
-          <t>회기역, 외대앞역</t>
+          <t>Hoegi Stn, ~15 min walk or bus to KHU</t>
         </is>
       </c>
       <c r="I32" s="4" t="inlineStr">
         <is>
-          <t>Hoegi Stn, ~15 min walk or bus to KHU</t>
-        </is>
-      </c>
-      <c r="J32" s="4" t="inlineStr">
-        <is>
           <t>Fridge, Washer, A/C, TV, WiFi, Gas range, Bed, all utilities included</t>
         </is>
       </c>
-      <c r="K32" s="4" t="inlineStr">
-        <is>
-          <t>Yes — English app, foreign card OK</t>
-        </is>
-      </c>
-      <c r="L32" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="M32" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="N32" s="4" t="inlineStr">
+      <c r="J32" s="5" t="inlineStr">
+        <is>
+          <t>Open link</t>
+        </is>
+      </c>
+      <c r="K32" s="5" t="inlineStr">
+        <is>
+          <t>Open link</t>
+        </is>
+      </c>
+      <c r="L32" s="4" t="inlineStr">
         <is>
           <t>Min 1 week. Short-stay OK. 관리비 ₩173,333/mo included in total.</t>
         </is>
@@ -2593,65 +2301,55 @@
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>33m2</t>
+          <t>Detached house</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>Detached house</t>
+          <t>₩823,333 / mo  (₩190,000 / week)</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>₩823,333 / mo  (₩190,000 / week)</t>
+          <t>₩1,126,666 / mo</t>
         </is>
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>₩1,126,666 / mo</t>
+          <t>₩330,000</t>
         </is>
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>₩330,000</t>
+          <t>23 m²</t>
         </is>
       </c>
       <c r="G33" s="4" t="inlineStr">
         <is>
-          <t>23 m²</t>
+          <t>회기역</t>
         </is>
       </c>
       <c r="H33" s="4" t="inlineStr">
         <is>
-          <t>회기역</t>
+          <t>Hoegi Stn, ~15 min walk or bus to KHU</t>
         </is>
       </c>
       <c r="I33" s="4" t="inlineStr">
         <is>
-          <t>Hoegi Stn, ~15 min walk or bus to KHU</t>
-        </is>
-      </c>
-      <c r="J33" s="4" t="inlineStr">
-        <is>
           <t>Fridge, Washer, A/C, WiFi, Induction, Bed, all utilities included</t>
         </is>
       </c>
-      <c r="K33" s="4" t="inlineStr">
-        <is>
-          <t>Yes — English app, foreign card OK</t>
-        </is>
-      </c>
-      <c r="L33" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="M33" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="N33" s="4" t="inlineStr">
+      <c r="J33" s="5" t="inlineStr">
+        <is>
+          <t>Open link</t>
+        </is>
+      </c>
+      <c r="K33" s="5" t="inlineStr">
+        <is>
+          <t>Open link</t>
+        </is>
+      </c>
+      <c r="L33" s="4" t="inlineStr">
         <is>
           <t>Min 2 weeks. Short-stay OK. 관리비 ₩303,333/mo included in total.</t>
         </is>
@@ -2665,65 +2363,55 @@
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>33m2</t>
+          <t>쉐어하우스</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>쉐어하우스</t>
+          <t>₩953,333 / mo  (₩220,000 / week)</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>₩953,333 / mo  (₩220,000 / week)</t>
+          <t>₩1,170,000 / mo</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>₩1,170,000 / mo</t>
+          <t>₩330,000</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>₩330,000</t>
+          <t>26 m²</t>
         </is>
       </c>
       <c r="G34" s="4" t="inlineStr">
         <is>
-          <t>26 m²</t>
+          <t>외대앞역, 회기역</t>
         </is>
       </c>
       <c r="H34" s="4" t="inlineStr">
         <is>
-          <t>외대앞역, 회기역</t>
+          <t>Hoegi Stn, ~15 min walk or bus to KHU</t>
         </is>
       </c>
       <c r="I34" s="4" t="inlineStr">
         <is>
-          <t>Hoegi Stn, ~15 min walk or bus to KHU</t>
-        </is>
-      </c>
-      <c r="J34" s="4" t="inlineStr">
-        <is>
           <t>Fridge, Washer, A/C, WiFi, Gas range, Bed, all utilities included</t>
         </is>
       </c>
-      <c r="K34" s="4" t="inlineStr">
-        <is>
-          <t>Yes — English app, foreign card OK</t>
-        </is>
-      </c>
-      <c r="L34" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="M34" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="N34" s="4" t="inlineStr">
+      <c r="J34" s="5" t="inlineStr">
+        <is>
+          <t>Open link</t>
+        </is>
+      </c>
+      <c r="K34" s="5" t="inlineStr">
+        <is>
+          <t>Open link</t>
+        </is>
+      </c>
+      <c r="L34" s="4" t="inlineStr">
         <is>
           <t>Min 1 week. Short-stay OK. 관리비 ₩216,667/mo included in total.</t>
         </is>
@@ -2731,66 +2419,66 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L5" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M5" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L6" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M6" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L7" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M7" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L8" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M8" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L9" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M9" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L10" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M10" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L11" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M11" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L12" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M12" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L13" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M13" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L14" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M14" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L15" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M15" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M16" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L17" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M17" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L18" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M18" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L19" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M19" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L20" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M20" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L21" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M21" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L22" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M22" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L23" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M23" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L24" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M24" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L25" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M25" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L26" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M26" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L27" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M27" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L28" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M28" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L29" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M29" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L30" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M30" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L31" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M31" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L32" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M32" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L33" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M33" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L34" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M34" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J5" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K5" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J6" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K6" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J7" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K8" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J9" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K9" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J10" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K10" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J11" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K11" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J12" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K12" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J13" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K13" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J14" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K14" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J15" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K15" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J16" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K16" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J17" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K17" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J18" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K18" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J19" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K19" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J20" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K20" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J21" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K21" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J22" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K22" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J23" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K23" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J24" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K24" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J25" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K25" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J26" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K26" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J27" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K27" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J28" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K28" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J29" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K29" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J30" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K30" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J31" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K31" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J32" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K32" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J33" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K33" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J34" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K34" r:id="rId60"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: scroll fade indicator + fix 쉐어하우스 filter spelling
- Add .table-outer wrapper with right-edge fade gradient + 'scroll ›' badge
- Badge/fade disappear when scrolled to end (JS scroll listener)
- Hidden on mobile (touch scroll is natural)
- Fix excluded type: add '쉐어하우스' (was only '셰어하우스'), 'Share house'
- listings now: Furnished studio + Detached house only (12 rooms ≤₩1.2M)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/rooms.xlsx
+++ b/rooms.xlsx
@@ -464,7 +464,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L34"/>
+  <dimension ref="A1:L16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -560,22 +560,22 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>외대,경희대풀옵2인실B</t>
+          <t>경희대 2분 풀옵션원룸</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>쉐어하우스</t>
+          <t>Furnished studio</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>₩498,333 / mo  (₩115,000 / week)</t>
+          <t>₩736,667 / mo  (₩170,000 / week)</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>₩585,000 / mo</t>
+          <t>₩736,667 / mo</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
@@ -590,7 +590,7 @@
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>회기역, 외대앞역</t>
+          <t>회기역</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
@@ -600,7 +600,7 @@
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>Fridge, Washer, A/C, WiFi, Induction, Bed, all utilities included</t>
+          <t>Fridge, Washer, A/C, WiFi, Gas range, Bed, all utilities included</t>
         </is>
       </c>
       <c r="J5" s="5" t="inlineStr">
@@ -615,29 +615,29 @@
       </c>
       <c r="L5" s="4" t="inlineStr">
         <is>
-          <t>Min 2 weeks. Short-stay OK. 관리비 ₩86,667/mo included in total.</t>
+          <t>Min 2 weeks. Short-stay OK.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>경희대외대시립대풀옵션A</t>
+          <t>깔끔 TV 비데 주차</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>쉐어하우스</t>
+          <t>Furnished studio</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>₩541,667 / mo  (₩125,000 / week)</t>
+          <t>₩736,667 / mo  (₩170,000 / week)</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>₩598,000 / mo</t>
+          <t>₩780,000 / mo</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
@@ -647,7 +647,7 @@
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>10 m²</t>
+          <t>17 m²</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
@@ -662,7 +662,7 @@
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>Fridge, Washer, A/C, TV, WiFi, Gas range, Bed, all utilities included</t>
+          <t>Fridge, Washer, A/C, TV, WiFi, Induction, Bed, water included</t>
         </is>
       </c>
       <c r="J6" s="5" t="inlineStr">
@@ -677,29 +677,29 @@
       </c>
       <c r="L6" s="4" t="inlineStr">
         <is>
-          <t>Min 12 weeks. 관리비 ₩56,333/mo included in total.</t>
+          <t>Min 2 weeks. Short-stay OK. 관리비 ₩43,333/mo included in total.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Room C-2</t>
+          <t>특가 🛎️ 외대2분 풀옵</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>쉐어하우스</t>
+          <t>Furnished studio</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>₩541,667 / mo  (₩125,000 / week)</t>
+          <t>₩780,000 / mo  (₩180,000 / week)</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>₩650,000 / mo</t>
+          <t>₩823,333 / mo</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
@@ -709,12 +709,12 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>17 m²</t>
+          <t>20 m²</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>회기역, 외대앞역</t>
+          <t>외대앞역, 회기역</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
@@ -739,29 +739,29 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Min 11 weeks. 관리비 ₩108,333/mo included in total.</t>
+          <t>Min 1 week. Short-stay OK. 관리비 ₩43,333/mo included in total.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>경희대회기역풀옵1인실C</t>
+          <t>회기역세권‼️B02😉</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>쉐어하우스</t>
+          <t>Detached house</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>₩520,000 / mo  (₩120,000 / week)</t>
+          <t>₩563,333 / mo  (₩130,000 / week)</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>₩650,000 / mo</t>
+          <t>₩866,666 / mo</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
@@ -771,7 +771,7 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>3 m²</t>
+          <t>13 m²</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
@@ -786,7 +786,7 @@
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>Fridge, Washer, A/C, WiFi, Gas range, Bed, all utilities included</t>
+          <t>Fridge, Washer, A/C, WiFi, Induction, Bed, all utilities included</t>
         </is>
       </c>
       <c r="J8" s="5" t="inlineStr">
@@ -801,29 +801,29 @@
       </c>
       <c r="L8" s="4" t="inlineStr">
         <is>
-          <t>Min 1 week. Short-stay OK. 관리비 ₩130,000/mo included in total.</t>
+          <t>Min 2 weeks. Short-stay OK. 관리비 ₩303,333/mo included in total.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>럭키하우스</t>
+          <t>외대역도보3분 경희대</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>쉐어하우스</t>
+          <t>Detached house</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>₩606,667 / mo  (₩140,000 / week)</t>
+          <t>₩866,667 / mo  (₩200,000 / week)</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>₩693,334 / mo</t>
+          <t>₩866,667 / mo</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
@@ -833,12 +833,12 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>20 m²</t>
+          <t>40 m²</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>회기역</t>
+          <t>회기역, 외대앞역</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
@@ -848,7 +848,7 @@
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>Fridge, Washer, A/C, WiFi, Gas range, Bed, all utilities included</t>
+          <t>Fridge, Washer, A/C, TV, Induction, Bed, all utilities included</t>
         </is>
       </c>
       <c r="J9" s="5" t="inlineStr">
@@ -863,29 +863,29 @@
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>Min 4 weeks. 관리비 ₩86,667/mo included in total.</t>
+          <t>Min 1 week. Short-stay OK.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>한국외대경희대풀옵션C</t>
+          <t>회기삼육 조용한 독채</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>쉐어하우스</t>
+          <t>Detached house</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>₩585,000 / mo  (₩135,000 / week)</t>
+          <t>₩736,667 / mo  (₩170,000 / week)</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>₩715,000 / mo</t>
+          <t>₩888,334 / mo</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
@@ -895,12 +895,12 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>13 m²</t>
+          <t>20 m²</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>회기역, 외대앞역</t>
+          <t>회기역</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
@@ -910,7 +910,7 @@
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>Fridge, Washer, A/C, TV, WiFi, Gas range, Bed, all utilities included</t>
+          <t>Fridge, Washer, A/C, Gas range, Bed, all utilities included</t>
         </is>
       </c>
       <c r="J10" s="5" t="inlineStr">
@@ -925,29 +925,29 @@
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>Min 2 weeks. Short-stay OK. 관리비 ₩130,000/mo included in total.</t>
+          <t>Min 1 week. Short-stay OK. 관리비 ₩151,667/mo included in total.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>Room B</t>
+          <t>아늑한방!!회기역8분</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>쉐어하우스</t>
+          <t>Detached house</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>₩628,333 / mo  (₩145,000 / week)</t>
+          <t>₩650,000 / mo  (₩150,000 / week)</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>₩736,666 / mo</t>
+          <t>₩953,333 / mo</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
@@ -957,12 +957,12 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>7 m²</t>
+          <t>17 m²</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>회기역, 외대앞역</t>
+          <t>회기역</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
@@ -972,7 +972,7 @@
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>Fridge, Washer, A/C, WiFi, Induction, Bed, all utilities included</t>
+          <t>Fridge, Washer, A/C, WiFi, Gas range, Bed, all utilities included</t>
         </is>
       </c>
       <c r="J11" s="5" t="inlineStr">
@@ -987,29 +987,29 @@
       </c>
       <c r="L11" s="4" t="inlineStr">
         <is>
-          <t>Min 11 weeks. 관리비 ₩108,333/mo included in total.</t>
+          <t>Min 2 weeks. Short-stay OK. 관리비 ₩303,333/mo included in total.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>경희대 2분 풀옵션원룸</t>
+          <t>특가😲‼️ 회기역세권</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Furnished studio</t>
+          <t>Detached house</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>₩736,667 / mo  (₩170,000 / week)</t>
+          <t>₩650,000 / mo  (₩150,000 / week)</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>₩736,667 / mo</t>
+          <t>₩953,333 / mo</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
@@ -1019,7 +1019,7 @@
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>13 m²</t>
+          <t>20 m²</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
@@ -1034,7 +1034,7 @@
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>Fridge, Washer, A/C, WiFi, Gas range, Bed, all utilities included</t>
+          <t>Fridge, Washer, A/C, WiFi, Induction, Bed, all utilities included</t>
         </is>
       </c>
       <c r="J12" s="5" t="inlineStr">
@@ -1049,29 +1049,29 @@
       </c>
       <c r="L12" s="4" t="inlineStr">
         <is>
-          <t>Min 2 weeks. Short-stay OK.</t>
+          <t>Min 2 weeks. Short-stay OK. 관리비 ₩303,333/mo included in total.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>외대,경희대풀옵1인실A</t>
+          <t>경희대2분 풀옵션원룸</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>쉐어하우스</t>
+          <t>Furnished studio</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>₩650,000 / mo  (₩150,000 / week)</t>
+          <t>₩953,333 / mo  (₩220,000 / week)</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>₩736,667 / mo</t>
+          <t>₩953,333 / mo</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
@@ -1081,12 +1081,12 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>10 m²</t>
+          <t>20 m²</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>회기역, 외대앞역</t>
+          <t>회기역</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
@@ -1096,7 +1096,7 @@
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>Fridge, Washer, A/C, WiFi, Induction, Bed, all utilities included</t>
+          <t>Fridge, Washer, A/C, WiFi, Gas range, Bed, all utilities included</t>
         </is>
       </c>
       <c r="J13" s="5" t="inlineStr">
@@ -1111,29 +1111,29 @@
       </c>
       <c r="L13" s="4" t="inlineStr">
         <is>
-          <t>Min 1 week. Short-stay OK. 관리비 ₩86,667/mo included in total.</t>
+          <t>Min 2 weeks. Short-stay OK.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>깔끔 TV 비데 주차</t>
+          <t>편안한방😋경희대3분!</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Furnished studio</t>
+          <t>Detached house</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>₩736,667 / mo  (₩170,000 / week)</t>
+          <t>₩693,333 / mo  (₩160,000 / week)</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>₩780,000 / mo</t>
+          <t>₩996,666 / mo</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
@@ -1143,12 +1143,12 @@
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>17 m²</t>
+          <t>20 m²</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>회기역, 외대앞역</t>
+          <t>회기역</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>Fridge, Washer, A/C, TV, WiFi, Induction, Bed, water included</t>
+          <t>Fridge, Washer, A/C, WiFi, Induction, Bed, all utilities included</t>
         </is>
       </c>
       <c r="J14" s="5" t="inlineStr">
@@ -1173,29 +1173,29 @@
       </c>
       <c r="L14" s="4" t="inlineStr">
         <is>
-          <t>Min 2 weeks. Short-stay OK. 관리비 ₩43,333/mo included in total.</t>
+          <t>Min 2 weeks. Short-stay OK. 관리비 ₩303,333/mo included in total.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>2인실A(창가쪽)</t>
+          <t>🎈회기역 도보3분 넓음</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>쉐어하우스</t>
+          <t>Furnished studio</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>₩650,000 / mo  (₩150,000 / week)</t>
+          <t>₩910,000 / mo  (₩210,000 / week)</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>₩780,000 / mo</t>
+          <t>₩1,083,333 / mo</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
@@ -1205,7 +1205,7 @@
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>13 m²</t>
+          <t>23 m²</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
@@ -1220,7 +1220,7 @@
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>Fridge, Washer, A/C, WiFi, Gas range, Induction, Bed, all utilities included</t>
+          <t>Fridge, Washer, A/C, TV, WiFi, Gas range, Bed, all utilities included</t>
         </is>
       </c>
       <c r="J15" s="5" t="inlineStr">
@@ -1235,29 +1235,29 @@
       </c>
       <c r="L15" s="4" t="inlineStr">
         <is>
-          <t>Min 1 week. Short-stay OK. 관리비 ₩130,000/mo included in total.</t>
+          <t>Min 1 week. Short-stay OK. 관리비 ₩173,333/mo included in total.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>경희대회기역풀옵2인실A</t>
+          <t>갬성있는방!!회기역8분</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>쉐어하우스</t>
+          <t>Detached house</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>₩650,000 / mo  (₩150,000 / week)</t>
+          <t>₩823,333 / mo  (₩190,000 / week)</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>₩780,000 / mo</t>
+          <t>₩1,126,666 / mo</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
@@ -1267,7 +1267,7 @@
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>7 m²</t>
+          <t>23 m²</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
@@ -1282,7 +1282,7 @@
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>Fridge, Washer, A/C, WiFi, Gas range, Bed, all utilities included</t>
+          <t>Fridge, Washer, A/C, WiFi, Induction, Bed, all utilities included</t>
         </is>
       </c>
       <c r="J16" s="5" t="inlineStr">
@@ -1297,1123 +1297,7 @@
       </c>
       <c r="L16" s="4" t="inlineStr">
         <is>
-          <t>Min 1 week. Short-stay OK. 관리비 ₩130,000/mo included in total.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>Room A</t>
-        </is>
-      </c>
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t>쉐어하우스</t>
-        </is>
-      </c>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t>₩693,333 / mo  (₩160,000 / week)</t>
-        </is>
-      </c>
-      <c r="D17" s="4" t="inlineStr">
-        <is>
-          <t>₩801,666 / mo</t>
-        </is>
-      </c>
-      <c r="E17" s="4" t="inlineStr">
-        <is>
-          <t>₩330,000</t>
-        </is>
-      </c>
-      <c r="F17" s="4" t="inlineStr">
-        <is>
-          <t>10 m²</t>
-        </is>
-      </c>
-      <c r="G17" s="4" t="inlineStr">
-        <is>
-          <t>회기역, 외대앞역</t>
-        </is>
-      </c>
-      <c r="H17" s="4" t="inlineStr">
-        <is>
-          <t>Hoegi Stn, ~15 min walk or bus to KHU</t>
-        </is>
-      </c>
-      <c r="I17" s="4" t="inlineStr">
-        <is>
-          <t>Fridge, Washer, A/C, WiFi, Induction, Bed, all utilities included</t>
-        </is>
-      </c>
-      <c r="J17" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="K17" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="L17" s="4" t="inlineStr">
-        <is>
-          <t>Min 11 weeks. 관리비 ₩108,333/mo included in total.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="4" t="inlineStr">
-        <is>
-          <t>특가 🛎️ 외대2분 풀옵</t>
-        </is>
-      </c>
-      <c r="B18" s="4" t="inlineStr">
-        <is>
-          <t>Furnished studio</t>
-        </is>
-      </c>
-      <c r="C18" s="4" t="inlineStr">
-        <is>
-          <t>₩780,000 / mo  (₩180,000 / week)</t>
-        </is>
-      </c>
-      <c r="D18" s="4" t="inlineStr">
-        <is>
-          <t>₩823,333 / mo</t>
-        </is>
-      </c>
-      <c r="E18" s="4" t="inlineStr">
-        <is>
-          <t>₩330,000</t>
-        </is>
-      </c>
-      <c r="F18" s="4" t="inlineStr">
-        <is>
-          <t>20 m²</t>
-        </is>
-      </c>
-      <c r="G18" s="4" t="inlineStr">
-        <is>
-          <t>외대앞역, 회기역</t>
-        </is>
-      </c>
-      <c r="H18" s="4" t="inlineStr">
-        <is>
-          <t>Hoegi Stn, ~15 min walk or bus to KHU</t>
-        </is>
-      </c>
-      <c r="I18" s="4" t="inlineStr">
-        <is>
-          <t>Fridge, Washer, A/C, WiFi, Induction, Bed, all utilities included</t>
-        </is>
-      </c>
-      <c r="J18" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="K18" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="L18" s="4" t="inlineStr">
-        <is>
-          <t>Min 1 week. Short-stay OK. 관리비 ₩43,333/mo included in total.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t>회기역세권‼️B02😉</t>
-        </is>
-      </c>
-      <c r="B19" s="4" t="inlineStr">
-        <is>
-          <t>Detached house</t>
-        </is>
-      </c>
-      <c r="C19" s="4" t="inlineStr">
-        <is>
-          <t>₩563,333 / mo  (₩130,000 / week)</t>
-        </is>
-      </c>
-      <c r="D19" s="4" t="inlineStr">
-        <is>
-          <t>₩866,666 / mo</t>
-        </is>
-      </c>
-      <c r="E19" s="4" t="inlineStr">
-        <is>
-          <t>₩330,000</t>
-        </is>
-      </c>
-      <c r="F19" s="4" t="inlineStr">
-        <is>
-          <t>13 m²</t>
-        </is>
-      </c>
-      <c r="G19" s="4" t="inlineStr">
-        <is>
-          <t>회기역</t>
-        </is>
-      </c>
-      <c r="H19" s="4" t="inlineStr">
-        <is>
-          <t>Hoegi Stn, ~15 min walk or bus to KHU</t>
-        </is>
-      </c>
-      <c r="I19" s="4" t="inlineStr">
-        <is>
-          <t>Fridge, Washer, A/C, WiFi, Induction, Bed, all utilities included</t>
-        </is>
-      </c>
-      <c r="J19" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="K19" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="L19" s="4" t="inlineStr">
-        <is>
           <t>Min 2 weeks. Short-stay OK. 관리비 ₩303,333/mo included in total.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="4" t="inlineStr">
-        <is>
-          <t>외대역도보3분 경희대</t>
-        </is>
-      </c>
-      <c r="B20" s="4" t="inlineStr">
-        <is>
-          <t>Detached house</t>
-        </is>
-      </c>
-      <c r="C20" s="4" t="inlineStr">
-        <is>
-          <t>₩866,667 / mo  (₩200,000 / week)</t>
-        </is>
-      </c>
-      <c r="D20" s="4" t="inlineStr">
-        <is>
-          <t>₩866,667 / mo</t>
-        </is>
-      </c>
-      <c r="E20" s="4" t="inlineStr">
-        <is>
-          <t>₩330,000</t>
-        </is>
-      </c>
-      <c r="F20" s="4" t="inlineStr">
-        <is>
-          <t>40 m²</t>
-        </is>
-      </c>
-      <c r="G20" s="4" t="inlineStr">
-        <is>
-          <t>회기역, 외대앞역</t>
-        </is>
-      </c>
-      <c r="H20" s="4" t="inlineStr">
-        <is>
-          <t>Hoegi Stn, ~15 min walk or bus to KHU</t>
-        </is>
-      </c>
-      <c r="I20" s="4" t="inlineStr">
-        <is>
-          <t>Fridge, Washer, A/C, TV, Induction, Bed, all utilities included</t>
-        </is>
-      </c>
-      <c r="J20" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="K20" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="L20" s="4" t="inlineStr">
-        <is>
-          <t>Min 1 week. Short-stay OK.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="4" t="inlineStr">
-        <is>
-          <t>외대풀옵션외대앞1분깨끗</t>
-        </is>
-      </c>
-      <c r="B21" s="4" t="inlineStr">
-        <is>
-          <t>쉐어하우스</t>
-        </is>
-      </c>
-      <c r="C21" s="4" t="inlineStr">
-        <is>
-          <t>₩650,000 / mo  (₩150,000 / week)</t>
-        </is>
-      </c>
-      <c r="D21" s="4" t="inlineStr">
-        <is>
-          <t>₩866,667 / mo</t>
-        </is>
-      </c>
-      <c r="E21" s="4" t="inlineStr">
-        <is>
-          <t>₩330,000</t>
-        </is>
-      </c>
-      <c r="F21" s="4" t="inlineStr">
-        <is>
-          <t>17 m²</t>
-        </is>
-      </c>
-      <c r="G21" s="4" t="inlineStr">
-        <is>
-          <t>외대앞역, 회기역</t>
-        </is>
-      </c>
-      <c r="H21" s="4" t="inlineStr">
-        <is>
-          <t>Hoegi Stn, ~15 min walk or bus to KHU</t>
-        </is>
-      </c>
-      <c r="I21" s="4" t="inlineStr">
-        <is>
-          <t>Fridge, Washer, A/C, WiFi, Gas range, Bed, all utilities included</t>
-        </is>
-      </c>
-      <c r="J21" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="K21" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="L21" s="4" t="inlineStr">
-        <is>
-          <t>Min 1 week. Short-stay OK. 관리비 ₩216,667/mo included in total.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="4" t="inlineStr">
-        <is>
-          <t>회기삼육 조용한 독채</t>
-        </is>
-      </c>
-      <c r="B22" s="4" t="inlineStr">
-        <is>
-          <t>Detached house</t>
-        </is>
-      </c>
-      <c r="C22" s="4" t="inlineStr">
-        <is>
-          <t>₩736,667 / mo  (₩170,000 / week)</t>
-        </is>
-      </c>
-      <c r="D22" s="4" t="inlineStr">
-        <is>
-          <t>₩888,334 / mo</t>
-        </is>
-      </c>
-      <c r="E22" s="4" t="inlineStr">
-        <is>
-          <t>₩330,000</t>
-        </is>
-      </c>
-      <c r="F22" s="4" t="inlineStr">
-        <is>
-          <t>20 m²</t>
-        </is>
-      </c>
-      <c r="G22" s="4" t="inlineStr">
-        <is>
-          <t>회기역</t>
-        </is>
-      </c>
-      <c r="H22" s="4" t="inlineStr">
-        <is>
-          <t>Hoegi Stn, ~15 min walk or bus to KHU</t>
-        </is>
-      </c>
-      <c r="I22" s="4" t="inlineStr">
-        <is>
-          <t>Fridge, Washer, A/C, Gas range, Bed, all utilities included</t>
-        </is>
-      </c>
-      <c r="J22" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="K22" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="L22" s="4" t="inlineStr">
-        <is>
-          <t>Min 1 week. Short-stay OK. 관리비 ₩151,667/mo included in total.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="4" t="inlineStr">
-        <is>
-          <t>1인실B</t>
-        </is>
-      </c>
-      <c r="B23" s="4" t="inlineStr">
-        <is>
-          <t>쉐어하우스</t>
-        </is>
-      </c>
-      <c r="C23" s="4" t="inlineStr">
-        <is>
-          <t>₩780,000 / mo  (₩180,000 / week)</t>
-        </is>
-      </c>
-      <c r="D23" s="4" t="inlineStr">
-        <is>
-          <t>₩910,000 / mo</t>
-        </is>
-      </c>
-      <c r="E23" s="4" t="inlineStr">
-        <is>
-          <t>₩330,000</t>
-        </is>
-      </c>
-      <c r="F23" s="4" t="inlineStr">
-        <is>
-          <t>7 m²</t>
-        </is>
-      </c>
-      <c r="G23" s="4" t="inlineStr">
-        <is>
-          <t>회기역, 외대앞역</t>
-        </is>
-      </c>
-      <c r="H23" s="4" t="inlineStr">
-        <is>
-          <t>Hoegi Stn, ~15 min walk or bus to KHU</t>
-        </is>
-      </c>
-      <c r="I23" s="4" t="inlineStr">
-        <is>
-          <t>Fridge, Washer, A/C, WiFi, Gas range, Induction, Bed, all utilities included</t>
-        </is>
-      </c>
-      <c r="J23" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="K23" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="L23" s="4" t="inlineStr">
-        <is>
-          <t>Min 1 week. Short-stay OK. 관리비 ₩130,000/mo included in total.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="4" t="inlineStr">
-        <is>
-          <t>아늑한방!!회기역8분</t>
-        </is>
-      </c>
-      <c r="B24" s="4" t="inlineStr">
-        <is>
-          <t>Detached house</t>
-        </is>
-      </c>
-      <c r="C24" s="4" t="inlineStr">
-        <is>
-          <t>₩650,000 / mo  (₩150,000 / week)</t>
-        </is>
-      </c>
-      <c r="D24" s="4" t="inlineStr">
-        <is>
-          <t>₩953,333 / mo</t>
-        </is>
-      </c>
-      <c r="E24" s="4" t="inlineStr">
-        <is>
-          <t>₩330,000</t>
-        </is>
-      </c>
-      <c r="F24" s="4" t="inlineStr">
-        <is>
-          <t>17 m²</t>
-        </is>
-      </c>
-      <c r="G24" s="4" t="inlineStr">
-        <is>
-          <t>회기역</t>
-        </is>
-      </c>
-      <c r="H24" s="4" t="inlineStr">
-        <is>
-          <t>Hoegi Stn, ~15 min walk or bus to KHU</t>
-        </is>
-      </c>
-      <c r="I24" s="4" t="inlineStr">
-        <is>
-          <t>Fridge, Washer, A/C, WiFi, Gas range, Bed, all utilities included</t>
-        </is>
-      </c>
-      <c r="J24" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="K24" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="L24" s="4" t="inlineStr">
-        <is>
-          <t>Min 2 weeks. Short-stay OK. 관리비 ₩303,333/mo included in total.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="4" t="inlineStr">
-        <is>
-          <t>특가😲‼️ 회기역세권</t>
-        </is>
-      </c>
-      <c r="B25" s="4" t="inlineStr">
-        <is>
-          <t>Detached house</t>
-        </is>
-      </c>
-      <c r="C25" s="4" t="inlineStr">
-        <is>
-          <t>₩650,000 / mo  (₩150,000 / week)</t>
-        </is>
-      </c>
-      <c r="D25" s="4" t="inlineStr">
-        <is>
-          <t>₩953,333 / mo</t>
-        </is>
-      </c>
-      <c r="E25" s="4" t="inlineStr">
-        <is>
-          <t>₩330,000</t>
-        </is>
-      </c>
-      <c r="F25" s="4" t="inlineStr">
-        <is>
-          <t>20 m²</t>
-        </is>
-      </c>
-      <c r="G25" s="4" t="inlineStr">
-        <is>
-          <t>회기역</t>
-        </is>
-      </c>
-      <c r="H25" s="4" t="inlineStr">
-        <is>
-          <t>Hoegi Stn, ~15 min walk or bus to KHU</t>
-        </is>
-      </c>
-      <c r="I25" s="4" t="inlineStr">
-        <is>
-          <t>Fridge, Washer, A/C, WiFi, Induction, Bed, all utilities included</t>
-        </is>
-      </c>
-      <c r="J25" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="K25" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="L25" s="4" t="inlineStr">
-        <is>
-          <t>Min 2 weeks. Short-stay OK. 관리비 ₩303,333/mo included in total.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="4" t="inlineStr">
-        <is>
-          <t>경희대2분 풀옵션원룸</t>
-        </is>
-      </c>
-      <c r="B26" s="4" t="inlineStr">
-        <is>
-          <t>Furnished studio</t>
-        </is>
-      </c>
-      <c r="C26" s="4" t="inlineStr">
-        <is>
-          <t>₩953,333 / mo  (₩220,000 / week)</t>
-        </is>
-      </c>
-      <c r="D26" s="4" t="inlineStr">
-        <is>
-          <t>₩953,333 / mo</t>
-        </is>
-      </c>
-      <c r="E26" s="4" t="inlineStr">
-        <is>
-          <t>₩330,000</t>
-        </is>
-      </c>
-      <c r="F26" s="4" t="inlineStr">
-        <is>
-          <t>20 m²</t>
-        </is>
-      </c>
-      <c r="G26" s="4" t="inlineStr">
-        <is>
-          <t>회기역</t>
-        </is>
-      </c>
-      <c r="H26" s="4" t="inlineStr">
-        <is>
-          <t>Hoegi Stn, ~15 min walk or bus to KHU</t>
-        </is>
-      </c>
-      <c r="I26" s="4" t="inlineStr">
-        <is>
-          <t>Fridge, Washer, A/C, WiFi, Gas range, Bed, all utilities included</t>
-        </is>
-      </c>
-      <c r="J26" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="K26" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="L26" s="4" t="inlineStr">
-        <is>
-          <t>Min 2 weeks. Short-stay OK.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="4" t="inlineStr">
-        <is>
-          <t>회기역2분/경희대/외대</t>
-        </is>
-      </c>
-      <c r="B27" s="4" t="inlineStr">
-        <is>
-          <t>쉐어하우스</t>
-        </is>
-      </c>
-      <c r="C27" s="4" t="inlineStr">
-        <is>
-          <t>₩975,000 / mo  (₩225,000 / week)</t>
-        </is>
-      </c>
-      <c r="D27" s="4" t="inlineStr">
-        <is>
-          <t>₩975,000 / mo</t>
-        </is>
-      </c>
-      <c r="E27" s="4" t="inlineStr">
-        <is>
-          <t>₩330,000</t>
-        </is>
-      </c>
-      <c r="F27" s="4" t="inlineStr">
-        <is>
-          <t>10 m²</t>
-        </is>
-      </c>
-      <c r="G27" s="4" t="inlineStr">
-        <is>
-          <t>회기역, 외대앞역</t>
-        </is>
-      </c>
-      <c r="H27" s="4" t="inlineStr">
-        <is>
-          <t>Hoegi Stn, ~15 min walk or bus to KHU</t>
-        </is>
-      </c>
-      <c r="I27" s="4" t="inlineStr">
-        <is>
-          <t>Fridge, Washer, A/C, WiFi, Induction, Bed, all utilities included</t>
-        </is>
-      </c>
-      <c r="J27" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="K27" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="L27" s="4" t="inlineStr">
-        <is>
-          <t>Min 1 week. Short-stay OK.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="4" t="inlineStr">
-        <is>
-          <t>편안한방😋경희대3분!</t>
-        </is>
-      </c>
-      <c r="B28" s="4" t="inlineStr">
-        <is>
-          <t>Detached house</t>
-        </is>
-      </c>
-      <c r="C28" s="4" t="inlineStr">
-        <is>
-          <t>₩693,333 / mo  (₩160,000 / week)</t>
-        </is>
-      </c>
-      <c r="D28" s="4" t="inlineStr">
-        <is>
-          <t>₩996,666 / mo</t>
-        </is>
-      </c>
-      <c r="E28" s="4" t="inlineStr">
-        <is>
-          <t>₩330,000</t>
-        </is>
-      </c>
-      <c r="F28" s="4" t="inlineStr">
-        <is>
-          <t>20 m²</t>
-        </is>
-      </c>
-      <c r="G28" s="4" t="inlineStr">
-        <is>
-          <t>회기역</t>
-        </is>
-      </c>
-      <c r="H28" s="4" t="inlineStr">
-        <is>
-          <t>Hoegi Stn, ~15 min walk or bus to KHU</t>
-        </is>
-      </c>
-      <c r="I28" s="4" t="inlineStr">
-        <is>
-          <t>Fridge, Washer, A/C, WiFi, Induction, Bed, all utilities included</t>
-        </is>
-      </c>
-      <c r="J28" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="K28" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="L28" s="4" t="inlineStr">
-        <is>
-          <t>Min 2 weeks. Short-stay OK. 관리비 ₩303,333/mo included in total.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="4" t="inlineStr">
-        <is>
-          <t>경희대외대여성쉐어2인실</t>
-        </is>
-      </c>
-      <c r="B29" s="4" t="inlineStr">
-        <is>
-          <t>쉐어하우스</t>
-        </is>
-      </c>
-      <c r="C29" s="4" t="inlineStr">
-        <is>
-          <t>₩866,667 / mo  (₩200,000 / week)</t>
-        </is>
-      </c>
-      <c r="D29" s="4" t="inlineStr">
-        <is>
-          <t>₩996,667 / mo</t>
-        </is>
-      </c>
-      <c r="E29" s="4" t="inlineStr">
-        <is>
-          <t>₩330,000</t>
-        </is>
-      </c>
-      <c r="F29" s="4" t="inlineStr">
-        <is>
-          <t>17 m²</t>
-        </is>
-      </c>
-      <c r="G29" s="4" t="inlineStr">
-        <is>
-          <t>회기역, 외대앞역</t>
-        </is>
-      </c>
-      <c r="H29" s="4" t="inlineStr">
-        <is>
-          <t>Hoegi Stn, ~15 min walk or bus to KHU</t>
-        </is>
-      </c>
-      <c r="I29" s="4" t="inlineStr">
-        <is>
-          <t>Fridge, Washer, A/C, WiFi, Gas range, Bed, all utilities included</t>
-        </is>
-      </c>
-      <c r="J29" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="K29" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="L29" s="4" t="inlineStr">
-        <is>
-          <t>Min 4 weeks. 관리비 ₩130,000/mo included in total.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="4" t="inlineStr">
-        <is>
-          <t>외대풀옵션외대앞1분깨끗</t>
-        </is>
-      </c>
-      <c r="B30" s="4" t="inlineStr">
-        <is>
-          <t>쉐어하우스</t>
-        </is>
-      </c>
-      <c r="C30" s="4" t="inlineStr">
-        <is>
-          <t>₩736,667 / mo  (₩170,000 / week)</t>
-        </is>
-      </c>
-      <c r="D30" s="4" t="inlineStr">
-        <is>
-          <t>₩996,667 / mo</t>
-        </is>
-      </c>
-      <c r="E30" s="4" t="inlineStr">
-        <is>
-          <t>₩330,000</t>
-        </is>
-      </c>
-      <c r="F30" s="4" t="inlineStr">
-        <is>
-          <t>17 m²</t>
-        </is>
-      </c>
-      <c r="G30" s="4" t="inlineStr">
-        <is>
-          <t>외대앞역, 회기역</t>
-        </is>
-      </c>
-      <c r="H30" s="4" t="inlineStr">
-        <is>
-          <t>Hoegi Stn, ~15 min walk or bus to KHU</t>
-        </is>
-      </c>
-      <c r="I30" s="4" t="inlineStr">
-        <is>
-          <t>Fridge, Washer, A/C, WiFi, Gas range, Bed, all utilities included</t>
-        </is>
-      </c>
-      <c r="J30" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="K30" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="L30" s="4" t="inlineStr">
-        <is>
-          <t>Min 1 week. Short-stay OK. 관리비 ₩260,000/mo included in total.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="4" t="inlineStr">
-        <is>
-          <t>1인실A</t>
-        </is>
-      </c>
-      <c r="B31" s="4" t="inlineStr">
-        <is>
-          <t>쉐어하우스</t>
-        </is>
-      </c>
-      <c r="C31" s="4" t="inlineStr">
-        <is>
-          <t>₩910,000 / mo  (₩210,000 / week)</t>
-        </is>
-      </c>
-      <c r="D31" s="4" t="inlineStr">
-        <is>
-          <t>₩1,040,000 / mo</t>
-        </is>
-      </c>
-      <c r="E31" s="4" t="inlineStr">
-        <is>
-          <t>₩330,000</t>
-        </is>
-      </c>
-      <c r="F31" s="4" t="inlineStr">
-        <is>
-          <t>10 m²</t>
-        </is>
-      </c>
-      <c r="G31" s="4" t="inlineStr">
-        <is>
-          <t>회기역, 외대앞역</t>
-        </is>
-      </c>
-      <c r="H31" s="4" t="inlineStr">
-        <is>
-          <t>Hoegi Stn, ~15 min walk or bus to KHU</t>
-        </is>
-      </c>
-      <c r="I31" s="4" t="inlineStr">
-        <is>
-          <t>Fridge, Washer, A/C, WiFi, Gas range, Induction, Bed, all utilities included</t>
-        </is>
-      </c>
-      <c r="J31" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="K31" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="L31" s="4" t="inlineStr">
-        <is>
-          <t>Min 1 week. Short-stay OK. 관리비 ₩130,000/mo included in total.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="4" t="inlineStr">
-        <is>
-          <t>🎈회기역 도보3분 넓음</t>
-        </is>
-      </c>
-      <c r="B32" s="4" t="inlineStr">
-        <is>
-          <t>Furnished studio</t>
-        </is>
-      </c>
-      <c r="C32" s="4" t="inlineStr">
-        <is>
-          <t>₩910,000 / mo  (₩210,000 / week)</t>
-        </is>
-      </c>
-      <c r="D32" s="4" t="inlineStr">
-        <is>
-          <t>₩1,083,333 / mo</t>
-        </is>
-      </c>
-      <c r="E32" s="4" t="inlineStr">
-        <is>
-          <t>₩330,000</t>
-        </is>
-      </c>
-      <c r="F32" s="4" t="inlineStr">
-        <is>
-          <t>23 m²</t>
-        </is>
-      </c>
-      <c r="G32" s="4" t="inlineStr">
-        <is>
-          <t>회기역, 외대앞역</t>
-        </is>
-      </c>
-      <c r="H32" s="4" t="inlineStr">
-        <is>
-          <t>Hoegi Stn, ~15 min walk or bus to KHU</t>
-        </is>
-      </c>
-      <c r="I32" s="4" t="inlineStr">
-        <is>
-          <t>Fridge, Washer, A/C, TV, WiFi, Gas range, Bed, all utilities included</t>
-        </is>
-      </c>
-      <c r="J32" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="K32" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="L32" s="4" t="inlineStr">
-        <is>
-          <t>Min 1 week. Short-stay OK. 관리비 ₩173,333/mo included in total.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="4" t="inlineStr">
-        <is>
-          <t>갬성있는방!!회기역8분</t>
-        </is>
-      </c>
-      <c r="B33" s="4" t="inlineStr">
-        <is>
-          <t>Detached house</t>
-        </is>
-      </c>
-      <c r="C33" s="4" t="inlineStr">
-        <is>
-          <t>₩823,333 / mo  (₩190,000 / week)</t>
-        </is>
-      </c>
-      <c r="D33" s="4" t="inlineStr">
-        <is>
-          <t>₩1,126,666 / mo</t>
-        </is>
-      </c>
-      <c r="E33" s="4" t="inlineStr">
-        <is>
-          <t>₩330,000</t>
-        </is>
-      </c>
-      <c r="F33" s="4" t="inlineStr">
-        <is>
-          <t>23 m²</t>
-        </is>
-      </c>
-      <c r="G33" s="4" t="inlineStr">
-        <is>
-          <t>회기역</t>
-        </is>
-      </c>
-      <c r="H33" s="4" t="inlineStr">
-        <is>
-          <t>Hoegi Stn, ~15 min walk or bus to KHU</t>
-        </is>
-      </c>
-      <c r="I33" s="4" t="inlineStr">
-        <is>
-          <t>Fridge, Washer, A/C, WiFi, Induction, Bed, all utilities included</t>
-        </is>
-      </c>
-      <c r="J33" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="K33" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="L33" s="4" t="inlineStr">
-        <is>
-          <t>Min 2 weeks. Short-stay OK. 관리비 ₩303,333/mo included in total.</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="4" t="inlineStr">
-        <is>
-          <t>외대앞1분풀옵션외대깔끔</t>
-        </is>
-      </c>
-      <c r="B34" s="4" t="inlineStr">
-        <is>
-          <t>쉐어하우스</t>
-        </is>
-      </c>
-      <c r="C34" s="4" t="inlineStr">
-        <is>
-          <t>₩953,333 / mo  (₩220,000 / week)</t>
-        </is>
-      </c>
-      <c r="D34" s="4" t="inlineStr">
-        <is>
-          <t>₩1,170,000 / mo</t>
-        </is>
-      </c>
-      <c r="E34" s="4" t="inlineStr">
-        <is>
-          <t>₩330,000</t>
-        </is>
-      </c>
-      <c r="F34" s="4" t="inlineStr">
-        <is>
-          <t>26 m²</t>
-        </is>
-      </c>
-      <c r="G34" s="4" t="inlineStr">
-        <is>
-          <t>외대앞역, 회기역</t>
-        </is>
-      </c>
-      <c r="H34" s="4" t="inlineStr">
-        <is>
-          <t>Hoegi Stn, ~15 min walk or bus to KHU</t>
-        </is>
-      </c>
-      <c r="I34" s="4" t="inlineStr">
-        <is>
-          <t>Fridge, Washer, A/C, WiFi, Gas range, Bed, all utilities included</t>
-        </is>
-      </c>
-      <c r="J34" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="K34" s="5" t="inlineStr">
-        <is>
-          <t>Open link</t>
-        </is>
-      </c>
-      <c r="L34" s="4" t="inlineStr">
-        <is>
-          <t>Min 1 week. Short-stay OK. 관리비 ₩216,667/mo included in total.</t>
         </is>
       </c>
     </row>
@@ -2443,42 +1327,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K15" r:id="rId22"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J16" r:id="rId23"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K16" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J17" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K17" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J18" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K18" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J19" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K19" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J20" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K20" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J21" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K21" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J22" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K22" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J23" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K23" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J24" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K24" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J25" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K25" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J26" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K26" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J27" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K27" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J28" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K28" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J29" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K29" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J30" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K30" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J31" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K31" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J32" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K32" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J33" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K33" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J34" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K34" r:id="rId60"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>